<commit_message>
Limit Leadoverzicht lookups to the route blocks
A lead taken out of a route was still found in the herverdeling table and
shown as planned on day 3; the lookups now stop above that table.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011FyXP9H3d6DgkgPRnXmUiU
</commit_message>
<xml_diff>
--- a/ade-door2door/ADE - Door2Door Route.xlsx
+++ b/ade-door2door/ADE - Door2Door Route.xlsx
@@ -1551,11 +1551,11 @@
         <v>10</v>
       </c>
       <c r="D5" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B5,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B5,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E5" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B5,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B5,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
       <c r="G5" s="4" t="s">
@@ -1577,11 +1577,11 @@
         <v>10</v>
       </c>
       <c r="D6" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B6,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B6,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E6" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B6,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B6,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
       <c r="G6" s="6" t="s">
@@ -1603,11 +1603,11 @@
         <v>10</v>
       </c>
       <c r="D7" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B7,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B7,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E7" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B7,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B7,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
       <c r="G7" s="7" t="s">
@@ -1629,11 +1629,11 @@
         <v>12</v>
       </c>
       <c r="D8" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B8,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B8,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E8" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B8,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B8,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
       <c r="G8" s="8" t="s">
@@ -1655,11 +1655,11 @@
         <v>14</v>
       </c>
       <c r="D9" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B9,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B9,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E9" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B9,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B9,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
       <c r="G9" s="9" t="s">
@@ -1681,11 +1681,11 @@
         <v>14</v>
       </c>
       <c r="D10" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B10,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B10,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E10" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B10,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B10,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -1700,11 +1700,11 @@
         <v>10</v>
       </c>
       <c r="D11" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B11,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B11,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E11" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B11,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B11,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -1719,11 +1719,11 @@
         <v>10</v>
       </c>
       <c r="D12" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B12,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B12,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E12" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B12,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B12,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -1738,11 +1738,11 @@
         <v>10</v>
       </c>
       <c r="D13" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B13,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B13,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E13" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B13,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B13,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -1757,11 +1757,11 @@
         <v>10</v>
       </c>
       <c r="D14" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B14,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B14,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E14" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B14,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B14,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -1776,11 +1776,11 @@
         <v>14</v>
       </c>
       <c r="D15" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B15,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B15,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E15" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B15,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B15,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -1795,11 +1795,11 @@
         <v>10</v>
       </c>
       <c r="D16" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B16,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B16,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E16" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B16,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B16,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -1814,11 +1814,11 @@
         <v>14</v>
       </c>
       <c r="D17" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B17,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B17,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E17" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B17,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B17,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -1833,11 +1833,11 @@
         <v>10</v>
       </c>
       <c r="D18" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B18,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B18,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E18" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B18,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B18,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -1852,11 +1852,11 @@
         <v>10</v>
       </c>
       <c r="D19" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B19,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B19,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Yasmijn + Steven</v>
       </c>
       <c r="E19" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B19,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B19,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -1871,11 +1871,11 @@
         <v>14</v>
       </c>
       <c r="D20" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B20,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B20,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E20" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B20,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B20,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
     </row>
@@ -1890,11 +1890,11 @@
         <v>10</v>
       </c>
       <c r="D21" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B21,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B21,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E21" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B21,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B21,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
     </row>
@@ -1909,11 +1909,11 @@
         <v>10</v>
       </c>
       <c r="D22" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B22,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B22,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E22" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B22,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B22,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
     </row>
@@ -1928,11 +1928,11 @@
         <v>12</v>
       </c>
       <c r="D23" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B23,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B23,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E23" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B23,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B23,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
     </row>
@@ -1947,11 +1947,11 @@
         <v>12</v>
       </c>
       <c r="D24" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B24,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B24,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E24" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B24,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B24,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
     </row>
@@ -1966,11 +1966,11 @@
         <v>12</v>
       </c>
       <c r="D25" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B25,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B25,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E25" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B25,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B25,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
     </row>
@@ -1985,11 +1985,11 @@
         <v>14</v>
       </c>
       <c r="D26" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B26,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B26,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E26" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B26,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B26,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
     </row>
@@ -2004,11 +2004,11 @@
         <v>12</v>
       </c>
       <c r="D27" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B27,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B27,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E27" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B27,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B27,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>1</v>
       </c>
     </row>
@@ -2023,11 +2023,11 @@
         <v>12</v>
       </c>
       <c r="D28" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B28,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B28,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E28" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B28,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B28,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -2042,11 +2042,11 @@
         <v>12</v>
       </c>
       <c r="D29" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B29,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B29,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E29" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B29,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B29,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -2061,11 +2061,11 @@
         <v>16</v>
       </c>
       <c r="D30" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B30,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B30,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E30" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B30,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B30,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -2080,11 +2080,11 @@
         <v>12</v>
       </c>
       <c r="D31" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B31,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B31,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E31" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B31,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B31,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -2099,11 +2099,11 @@
         <v>12</v>
       </c>
       <c r="D32" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B32,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B32,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E32" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B32,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B32,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -2118,11 +2118,11 @@
         <v>12</v>
       </c>
       <c r="D33" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B33,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B33,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E33" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B33,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B33,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -2137,11 +2137,11 @@
         <v>12</v>
       </c>
       <c r="D34" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B34,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B34,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E34" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B34,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B34,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -2156,11 +2156,11 @@
         <v>12</v>
       </c>
       <c r="D35" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B35,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B35,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E35" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B35,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B35,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -2175,11 +2175,11 @@
         <v>12</v>
       </c>
       <c r="D36" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B36,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B36,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E36" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B36,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B36,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -2194,11 +2194,11 @@
         <v>12</v>
       </c>
       <c r="D37" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B37,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B37,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E37" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B37,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B37,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>2</v>
       </c>
     </row>
@@ -2213,11 +2213,11 @@
         <v>12</v>
       </c>
       <c r="D38" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B38,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B38,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E38" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B38,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B38,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -2232,11 +2232,11 @@
         <v>10</v>
       </c>
       <c r="D39" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B39,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B39,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E39" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B39,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B39,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -2251,11 +2251,11 @@
         <v>12</v>
       </c>
       <c r="D40" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B40,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B40,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E40" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B40,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B40,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -2270,11 +2270,11 @@
         <v>12</v>
       </c>
       <c r="D41" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B41,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B41,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E41" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B41,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B41,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -2289,11 +2289,11 @@
         <v>10</v>
       </c>
       <c r="D42" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B42,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B42,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E42" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B42,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B42,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -2308,11 +2308,11 @@
         <v>10</v>
       </c>
       <c r="D43" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B43,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B43,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E43" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B43,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B43,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -2327,11 +2327,11 @@
         <v>12</v>
       </c>
       <c r="D44" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B44,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B44,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E44" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B44,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B44,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -2346,11 +2346,11 @@
         <v>16</v>
       </c>
       <c r="D45" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B45,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B45,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E45" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B45,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B45,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -2365,11 +2365,11 @@
         <v>12</v>
       </c>
       <c r="D46" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B46,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B46,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E46" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B46,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B46,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>
@@ -2384,11 +2384,11 @@
         <v>14</v>
       </c>
       <c r="D47" s="0" t="str">
-        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B47,'Planning 2 teams'!$C$1:$C$300,0)),"Niet ingepland")</f>
+        <f aca="false">IFERROR(INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B47,'Planning 2 teams'!$C$1:$C$86,0)),"Niet ingepland")</f>
         <v>Friso + Thierry</v>
       </c>
       <c r="E47" s="0" t="n">
-        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$300,MATCH(B47,'Planning 2 teams'!$C$1:$C$300,0)),"DAG *"),"")</f>
+        <f aca="false">IFERROR(COUNTIF('Planning 2 teams'!$A$1:INDEX('Planning 2 teams'!$A$1:$A$86,MATCH(B47,'Planning 2 teams'!$C$1:$C$86,0)),"DAG *"),"")</f>
         <v>3</v>
       </c>
     </row>

</xml_diff>